<commit_message>
Add Excel intake template with sample data
</commit_message>
<xml_diff>
--- a/data/Master_Input_Reference_Data.xlsx
+++ b/data/Master_Input_Reference_Data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/779845864bfe6eeb/Desktop/LAB Product/Enterprise AI Adoption/Input Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\avims\AviProjects\enterprise-ai-adoption-platform\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="11_F25DC773A252ABDACC10486CA19B7CA45ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E1CF263-EC82-4718-BE20-67BED23A12AC}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF973DF1-2ED8-4756-9597-669AF7F1A4B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -218,7 +218,7 @@
     <t>AI Ethics Committee</t>
   </si>
   <si>
-    <t>Northgate Financial Services</t>
+    <t>Meridian Capital Advisors(Fictional Demo)</t>
   </si>
 </sst>
 </file>
@@ -372,6 +372,30 @@
   </cellStyles>
   <dxfs count="13">
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -595,30 +619,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -632,34 +632,30 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B0159720-8A65-4190-9498-AAF1570DF5E3}" name="Table1" displayName="Table1" ref="B3:C12" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B0159720-8A65-4190-9498-AAF1570DF5E3}" name="Table1" displayName="Table1" ref="B3:C12" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10" totalsRowBorderDxfId="9">
   <autoFilter ref="B3:C12" xr:uid="{B0159720-8A65-4190-9498-AAF1570DF5E3}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{950FD2E3-DD47-493D-8ACC-7A81688EBE74}" name="Category" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{89A8CB5E-DA21-4CB8-A142-7FF268909D8A}" name="Current State" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{950FD2E3-DD47-493D-8ACC-7A81688EBE74}" name="Category" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{89A8CB5E-DA21-4CB8-A142-7FF268909D8A}" name="Current State" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8A5E99F8-87AB-4A21-801C-A27490054115}" name="Table2" displayName="Table2" ref="B2:C16" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8A5E99F8-87AB-4A21-801C-A27490054115}" name="Table2" displayName="Table2" ref="B2:C16" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5" tableBorderDxfId="4" totalsRowBorderDxfId="3">
   <autoFilter ref="B2:C16" xr:uid="{8A5E99F8-87AB-4A21-801C-A27490054115}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7B7130F9-9EA5-444D-843B-976EA7411D38}" name="Category" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{72EB8B9E-4A04-4853-83D8-D47DCFE6ABD6}" name="Current State" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{7B7130F9-9EA5-444D-843B-976EA7411D38}" name="Category" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{72EB8B9E-4A04-4853-83D8-D47DCFE6ABD6}" name="Current State" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B1A4F44C-6FF5-430D-8B38-CE872B16B226}" name="Table3" displayName="Table3" ref="B3:C10" totalsRowShown="0" headerRowDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{B1A4F44C-6FF5-430D-8B38-CE872B16B226}" name="Table3" displayName="Table3" ref="B3:C10" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="B3:C10" xr:uid="{B1A4F44C-6FF5-430D-8B38-CE872B16B226}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{E6A13A74-A134-43CC-B646-8C168C5B8788}" name="Category"/>

</xml_diff>